<commit_message>
complete parse and check of Array Express data
</commit_message>
<xml_diff>
--- a/data/NMD_Perturbation_TopStudySamples_20260716.xlsx
+++ b/data/NMD_Perturbation_TopStudySamples_20260716.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://moffitt-my.sharepoint.com/personal/alyssa_obermayer_moffitt_org/Documents/Documents/Projects/Active/Public_NMD_Perturbation_Data/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\aobermayer4\Projects\active\Public_NMD_Perturbation_Data\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="49" documentId="8_{2499766E-EB53-4B85-8092-AE05928BB4F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{17491179-3172-4D53-A601-604A3C0209B1}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{434A45E9-96F9-4FDC-A7F4-2F27C1815340}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{DAD5C51E-F1D3-4296-A2F1-A74013D7D8F0}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="2" xr2:uid="{DAD5C51E-F1D3-4296-A2F1-A74013D7D8F0}"/>
   </bookViews>
   <sheets>
     <sheet name="NMD_Perturbation_TopStudySample" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2427" uniqueCount="913">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2485" uniqueCount="932">
   <si>
     <t>GSE_ID</t>
   </si>
@@ -2235,9 +2235,6 @@
     <t>UPF3A-UPF3B double knockout clone 1, wild type genotype, UPF3B knockout clone 90, UPF3A-UPF3B double knockout clone 2</t>
   </si>
   <si>
-    <t>Luciferase siRNA, UPF3B siRNA</t>
-  </si>
-  <si>
     <t>wild type genotype, SMG7 knockout clone 34, SMG7 knockout clone 2</t>
   </si>
   <si>
@@ -2761,6 +2758,66 @@
   </si>
   <si>
     <t>https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSE232333</t>
+  </si>
+  <si>
+    <t>Flp-In-T-REx-293</t>
+  </si>
+  <si>
+    <t>SMG5 siRNA, SMG6 siRNA</t>
+  </si>
+  <si>
+    <t>Luciferase siRNA, UPF3B siRNA, Also using UPF3B/UPFsA KO clones?</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>HCT116</t>
+  </si>
+  <si>
+    <t>?</t>
+  </si>
+  <si>
+    <t>24?</t>
+  </si>
+  <si>
+    <t>Flp-In-T-REx-U2OS</t>
+  </si>
+  <si>
+    <t>SMG8/SMG9 KO, not sure about siRNA or other method</t>
+  </si>
+  <si>
+    <t>SMG8/SMG9 KO or del, not sure about siRNA or other method</t>
+  </si>
+  <si>
+    <t>UPF1?</t>
+  </si>
+  <si>
+    <t>TERT-HFF</t>
+  </si>
+  <si>
+    <t>HUVEC/TERT 2</t>
+  </si>
+  <si>
+    <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC8233366/</t>
+  </si>
+  <si>
+    <t>we uncover that the loss of the first SMG5-SMG7-dependent pathway also inactivates the second SMG6-dependent branch, indicating an unexpected functional connection between the final NMD steps</t>
+  </si>
+  <si>
+    <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC9108619</t>
+  </si>
+  <si>
+    <t>UPF3B siRNA, UPF3A siRNA</t>
+  </si>
+  <si>
+    <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC7470949/</t>
+  </si>
+  <si>
+    <t>siRNAs were targeted against Luciferase, EIF4A3, RBM8A, CASC3, UPF1, XRN1, SMG6 or SMG7</t>
+  </si>
+  <si>
+    <t>perturbation samples might be with protein data</t>
   </si>
 </sst>
 </file>
@@ -3309,7 +3366,7 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
@@ -3329,6 +3386,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="42" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3709,37 +3769,37 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E28C8A8-6FB1-4F0E-BBCF-A1462531D658}">
   <dimension ref="A1:AE80"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="6" width="32.5703125" customWidth="1"/>
-    <col min="7" max="7" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.42578125" customWidth="1"/>
-    <col min="10" max="12" width="20.85546875" customWidth="1"/>
-    <col min="13" max="13" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="20.85546875" customWidth="1"/>
+    <col min="1" max="1" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="6" width="32.5546875" customWidth="1"/>
+    <col min="7" max="7" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.44140625" customWidth="1"/>
+    <col min="10" max="12" width="20.88671875" customWidth="1"/>
+    <col min="13" max="13" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="20.88671875" customWidth="1"/>
     <col min="16" max="16" width="8" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="24.140625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="26.42578125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="23.7109375" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="23.85546875" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="23.7109375" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="25.85546875" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="20.85546875" customWidth="1"/>
-    <col min="28" max="28" width="23.85546875" customWidth="1"/>
-    <col min="29" max="29" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="19.5703125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="20.85546875" customWidth="1"/>
+    <col min="17" max="17" width="24.109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="26.44140625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="23.88671875" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="25.88671875" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="20.88671875" customWidth="1"/>
+    <col min="28" max="28" width="23.88671875" customWidth="1"/>
+    <col min="29" max="29" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="19.5546875" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="20.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3831,7 +3891,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>28</v>
       </c>
@@ -3926,7 +3986,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>28</v>
       </c>
@@ -4021,7 +4081,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="4" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>28</v>
       </c>
@@ -4116,7 +4176,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="5" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>28</v>
       </c>
@@ -4211,7 +4271,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="6" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>28</v>
       </c>
@@ -4306,7 +4366,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="7" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>28</v>
       </c>
@@ -4401,7 +4461,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="8" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>28</v>
       </c>
@@ -4496,7 +4556,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="9" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>73</v>
       </c>
@@ -4591,7 +4651,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="10" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>73</v>
       </c>
@@ -4686,7 +4746,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="11" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>73</v>
       </c>
@@ -4781,7 +4841,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="12" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>73</v>
       </c>
@@ -4876,7 +4936,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="13" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
         <v>73</v>
       </c>
@@ -4971,7 +5031,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="14" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
         <v>73</v>
       </c>
@@ -5066,7 +5126,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="15" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
         <v>73</v>
       </c>
@@ -5161,7 +5221,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="16" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
         <v>73</v>
       </c>
@@ -5256,7 +5316,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="17" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
         <v>73</v>
       </c>
@@ -5351,7 +5411,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="18" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
         <v>73</v>
       </c>
@@ -5446,7 +5506,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="19" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
         <v>73</v>
       </c>
@@ -5541,7 +5601,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="20" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A20" s="3" t="s">
         <v>73</v>
       </c>
@@ -5636,7 +5696,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="21" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
         <v>73</v>
       </c>
@@ -5731,7 +5791,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="22" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
         <v>73</v>
       </c>
@@ -5826,7 +5886,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="23" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
         <v>73</v>
       </c>
@@ -5921,7 +5981,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="24" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
         <v>73</v>
       </c>
@@ -6016,7 +6076,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="25" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
         <v>73</v>
       </c>
@@ -6111,7 +6171,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="26" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A26" s="3" t="s">
         <v>73</v>
       </c>
@@ -6206,7 +6266,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="27" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
         <v>150</v>
       </c>
@@ -6298,7 +6358,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="28" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
         <v>150</v>
       </c>
@@ -6390,7 +6450,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="29" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
         <v>150</v>
       </c>
@@ -6482,7 +6542,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="30" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
         <v>150</v>
       </c>
@@ -6574,7 +6634,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="31" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
         <v>150</v>
       </c>
@@ -6666,7 +6726,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="32" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
         <v>150</v>
       </c>
@@ -6758,7 +6818,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="33" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A33" s="4" t="s">
         <v>150</v>
       </c>
@@ -6850,7 +6910,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="34" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
         <v>150</v>
       </c>
@@ -6942,7 +7002,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="35" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A35" s="4" t="s">
         <v>150</v>
       </c>
@@ -7034,7 +7094,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="36" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
         <v>150</v>
       </c>
@@ -7126,7 +7186,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="37" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A37" s="4" t="s">
         <v>150</v>
       </c>
@@ -7218,7 +7278,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="38" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
         <v>150</v>
       </c>
@@ -7310,7 +7370,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="39" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A39" s="4" t="s">
         <v>150</v>
       </c>
@@ -7402,7 +7462,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="40" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A40" s="4" t="s">
         <v>150</v>
       </c>
@@ -7494,7 +7554,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="41" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
         <v>206</v>
       </c>
@@ -7586,7 +7646,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="42" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
         <v>206</v>
       </c>
@@ -7678,7 +7738,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="43" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
         <v>206</v>
       </c>
@@ -7770,7 +7830,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="44" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
         <v>206</v>
       </c>
@@ -7862,7 +7922,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="45" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
         <v>206</v>
       </c>
@@ -7954,7 +8014,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="46" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
         <v>206</v>
       </c>
@@ -8046,7 +8106,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="47" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
         <v>206</v>
       </c>
@@ -8138,7 +8198,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="48" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
         <v>206</v>
       </c>
@@ -8230,7 +8290,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="49" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
         <v>206</v>
       </c>
@@ -8322,7 +8382,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="50" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
         <v>206</v>
       </c>
@@ -8414,7 +8474,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="51" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
         <v>206</v>
       </c>
@@ -8506,7 +8566,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="52" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
         <v>206</v>
       </c>
@@ -8598,7 +8658,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="53" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
         <v>206</v>
       </c>
@@ -8690,7 +8750,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="54" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
         <v>206</v>
       </c>
@@ -8782,7 +8842,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="55" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
         <v>206</v>
       </c>
@@ -8874,7 +8934,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="56" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
         <v>206</v>
       </c>
@@ -8966,7 +9026,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="57" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
         <v>206</v>
       </c>
@@ -9058,7 +9118,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="58" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
         <v>206</v>
       </c>
@@ -9150,7 +9210,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="59" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
         <v>206</v>
       </c>
@@ -9242,7 +9302,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="60" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
         <v>206</v>
       </c>
@@ -9334,7 +9394,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="61" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A61" s="5" t="s">
         <v>311</v>
       </c>
@@ -9429,7 +9489,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="62" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A62" s="5" t="s">
         <v>311</v>
       </c>
@@ -9524,7 +9584,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="63" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A63" s="5" t="s">
         <v>311</v>
       </c>
@@ -9619,7 +9679,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="64" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A64" s="5" t="s">
         <v>311</v>
       </c>
@@ -9714,7 +9774,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="65" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A65" s="5" t="s">
         <v>311</v>
       </c>
@@ -9809,7 +9869,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="66" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A66" s="5" t="s">
         <v>311</v>
       </c>
@@ -9904,7 +9964,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="67" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A67" s="5" t="s">
         <v>311</v>
       </c>
@@ -9999,7 +10059,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="68" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A68" s="5" t="s">
         <v>311</v>
       </c>
@@ -10094,7 +10154,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="69" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A69" s="5" t="s">
         <v>311</v>
       </c>
@@ -10189,7 +10249,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="70" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A70" s="5" t="s">
         <v>311</v>
       </c>
@@ -10284,7 +10344,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="71" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A71" s="5" t="s">
         <v>311</v>
       </c>
@@ -10379,7 +10439,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="72" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A72" s="5" t="s">
         <v>311</v>
       </c>
@@ -10474,7 +10534,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="73" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A73" s="6" t="s">
         <v>348</v>
       </c>
@@ -10566,7 +10626,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="74" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A74" s="6" t="s">
         <v>348</v>
       </c>
@@ -10655,7 +10715,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="75" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A75" s="6" t="s">
         <v>348</v>
       </c>
@@ -10744,7 +10804,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="76" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A76" s="6" t="s">
         <v>348</v>
       </c>
@@ -10833,7 +10893,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="77" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A77" s="6" t="s">
         <v>348</v>
       </c>
@@ -10925,7 +10985,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="78" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A78" s="6" t="s">
         <v>348</v>
       </c>
@@ -11014,7 +11074,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="79" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A79" s="6" t="s">
         <v>348</v>
       </c>
@@ -11103,7 +11163,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="80" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A80" s="6" t="s">
         <v>348</v>
       </c>
@@ -11200,21 +11260,21 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA1739B9-C94C-4465-8F8F-0F3F742A5026}">
   <dimension ref="A1:R87"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="24.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="28.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.7109375" customWidth="1"/>
-    <col min="5" max="5" width="44.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="21.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="79.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="18" width="16.28515625" customWidth="1"/>
+    <col min="1" max="1" width="24.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.6640625" customWidth="1"/>
+    <col min="5" max="5" width="44.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="79.109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="18" width="16.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -11270,7 +11330,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>28</v>
       </c>
@@ -11320,7 +11380,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>73</v>
       </c>
@@ -11364,7 +11424,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>150</v>
       </c>
@@ -11414,7 +11474,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>457</v>
       </c>
@@ -11464,7 +11524,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>461</v>
       </c>
@@ -11514,7 +11574,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>206</v>
       </c>
@@ -11567,7 +11627,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>311</v>
       </c>
@@ -11620,7 +11680,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>348</v>
       </c>
@@ -11667,7 +11727,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A10" s="7" t="s">
         <v>469</v>
       </c>
@@ -11717,7 +11777,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>474</v>
       </c>
@@ -11764,7 +11824,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A12" s="7" t="s">
         <v>478</v>
       </c>
@@ -11817,7 +11877,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A13" s="7" t="s">
         <v>483</v>
       </c>
@@ -11861,7 +11921,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>487</v>
       </c>
@@ -11905,7 +11965,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>492</v>
       </c>
@@ -11949,7 +12009,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>497</v>
       </c>
@@ -11996,7 +12056,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>501</v>
       </c>
@@ -12043,7 +12103,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>505</v>
       </c>
@@ -12087,7 +12147,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>508</v>
       </c>
@@ -12134,7 +12194,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>513</v>
       </c>
@@ -12178,7 +12238,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>516</v>
       </c>
@@ -12222,7 +12282,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>519</v>
       </c>
@@ -12266,7 +12326,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>522</v>
       </c>
@@ -12310,7 +12370,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>524</v>
       </c>
@@ -12357,7 +12417,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>526</v>
       </c>
@@ -12401,7 +12461,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A26" s="7" t="s">
         <v>529</v>
       </c>
@@ -12451,7 +12511,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>532</v>
       </c>
@@ -12492,7 +12552,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="28" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>535</v>
       </c>
@@ -12539,7 +12599,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="29" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>539</v>
       </c>
@@ -12583,7 +12643,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="30" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>542</v>
       </c>
@@ -12627,7 +12687,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="31" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>545</v>
       </c>
@@ -12671,7 +12731,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="32" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>548</v>
       </c>
@@ -12715,7 +12775,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>551</v>
       </c>
@@ -12726,7 +12786,7 @@
         <v>553</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>554</v>
       </c>
@@ -12737,7 +12797,7 @@
         <v>556</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>557</v>
       </c>
@@ -12748,7 +12808,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>560</v>
       </c>
@@ -12759,7 +12819,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>563</v>
       </c>
@@ -12770,7 +12830,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>565</v>
       </c>
@@ -12781,7 +12841,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>567</v>
       </c>
@@ -12792,7 +12852,7 @@
         <v>569</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>570</v>
       </c>
@@ -12803,7 +12863,7 @@
         <v>572</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>573</v>
       </c>
@@ -12814,7 +12874,7 @@
         <v>575</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>576</v>
       </c>
@@ -12825,7 +12885,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>579</v>
       </c>
@@ -12836,7 +12896,7 @@
         <v>581</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>582</v>
       </c>
@@ -12847,7 +12907,7 @@
         <v>584</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>585</v>
       </c>
@@ -12858,7 +12918,7 @@
         <v>587</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>588</v>
       </c>
@@ -12869,7 +12929,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>591</v>
       </c>
@@ -12880,7 +12940,7 @@
         <v>593</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>594</v>
       </c>
@@ -12891,7 +12951,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>596</v>
       </c>
@@ -12902,7 +12962,7 @@
         <v>597</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>598</v>
       </c>
@@ -12913,7 +12973,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>600</v>
       </c>
@@ -12924,7 +12984,7 @@
         <v>601</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>602</v>
       </c>
@@ -12935,7 +12995,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>604</v>
       </c>
@@ -12946,7 +13006,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>606</v>
       </c>
@@ -12957,7 +13017,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>608</v>
       </c>
@@ -12968,7 +13028,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>610</v>
       </c>
@@ -12979,7 +13039,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A59" s="9" t="s">
         <v>612</v>
       </c>
@@ -12996,7 +13056,7 @@
         <v>616</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A60" s="9" t="s">
         <v>617</v>
       </c>
@@ -13013,7 +13073,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A61" s="9" t="s">
         <v>621</v>
       </c>
@@ -13030,7 +13090,7 @@
         <v>624</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A62" s="9" t="s">
         <v>625</v>
       </c>
@@ -13047,7 +13107,7 @@
         <v>628</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A63" s="10" t="s">
         <v>629</v>
       </c>
@@ -13064,7 +13124,7 @@
         <v>632</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A64" s="9" t="s">
         <v>633</v>
       </c>
@@ -13081,7 +13141,7 @@
         <v>636</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A65" s="10" t="s">
         <v>637</v>
       </c>
@@ -13098,7 +13158,7 @@
         <v>640</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A66" s="10" t="s">
         <v>641</v>
       </c>
@@ -13115,7 +13175,7 @@
         <v>644</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A67" s="10" t="s">
         <v>645</v>
       </c>
@@ -13132,7 +13192,7 @@
         <v>648</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A68" s="10" t="s">
         <v>649</v>
       </c>
@@ -13149,7 +13209,7 @@
         <v>652</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A69" s="10" t="s">
         <v>653</v>
       </c>
@@ -13166,7 +13226,7 @@
         <v>656</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A70" s="10" t="s">
         <v>657</v>
       </c>
@@ -13183,7 +13243,7 @@
         <v>660</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A71" s="10" t="s">
         <v>661</v>
       </c>
@@ -13200,7 +13260,7 @@
         <v>664</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A72" s="10" t="s">
         <v>665</v>
       </c>
@@ -13217,7 +13277,7 @@
         <v>668</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A73" s="10" t="s">
         <v>669</v>
       </c>
@@ -13234,7 +13294,7 @@
         <v>672</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A74" s="10" t="s">
         <v>669</v>
       </c>
@@ -13251,7 +13311,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A75" s="10" t="s">
         <v>675</v>
       </c>
@@ -13268,7 +13328,7 @@
         <v>678</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A76" s="10" t="s">
         <v>679</v>
       </c>
@@ -13285,7 +13345,7 @@
         <v>682</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A77" s="10" t="s">
         <v>683</v>
       </c>
@@ -13302,7 +13362,7 @@
         <v>686</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A78" s="10" t="s">
         <v>683</v>
       </c>
@@ -13319,7 +13379,7 @@
         <v>688</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A79" s="10" t="s">
         <v>33</v>
       </c>
@@ -13336,7 +13396,7 @@
         <v>691</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A80" s="10" t="s">
         <v>33</v>
       </c>
@@ -13353,7 +13413,7 @@
         <v>692</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A81" s="10" t="s">
         <v>33</v>
       </c>
@@ -13370,7 +13430,7 @@
         <v>693</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A82" s="10" t="s">
         <v>33</v>
       </c>
@@ -13387,7 +13447,7 @@
         <v>694</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A83" s="10" t="s">
         <v>695</v>
       </c>
@@ -13404,7 +13464,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A84" s="10" t="s">
         <v>695</v>
       </c>
@@ -13421,7 +13481,7 @@
         <v>702</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A85" s="10" t="s">
         <v>703</v>
       </c>
@@ -13438,7 +13498,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A86" s="10" t="s">
         <v>708</v>
       </c>
@@ -13455,7 +13515,7 @@
         <v>712</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A87" s="10" t="s">
         <v>713</v>
       </c>
@@ -13480,27 +13540,27 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89C31724-8146-4D7C-A3D2-DC7D492096E6}">
   <dimension ref="A1:Q40"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.42578125" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.44140625" customWidth="1"/>
+    <col min="7" max="7" width="10.109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="9" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.7109375" style="13" customWidth="1"/>
-    <col min="12" max="12" width="66.85546875" style="13" customWidth="1"/>
-    <col min="14" max="14" width="11.140625" style="13" customWidth="1"/>
-    <col min="15" max="15" width="21.85546875" style="13" customWidth="1"/>
-    <col min="16" max="16" width="42.85546875" style="13" customWidth="1"/>
-    <col min="17" max="17" width="130.5703125" style="13" customWidth="1"/>
+    <col min="9" max="9" width="8.88671875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.6640625" style="13" customWidth="1"/>
+    <col min="12" max="12" width="66.88671875" style="13" customWidth="1"/>
+    <col min="14" max="14" width="11.109375" style="13" customWidth="1"/>
+    <col min="15" max="15" width="21.88671875" style="13" customWidth="1"/>
+    <col min="16" max="16" width="42.88671875" style="13" customWidth="1"/>
+    <col min="17" max="17" width="130.5546875" style="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>718</v>
       </c>
@@ -13529,45 +13589,45 @@
         <v>726</v>
       </c>
       <c r="J1" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="K1" s="13" t="s">
+        <v>772</v>
+      </c>
+      <c r="L1" s="13" t="s">
         <v>773</v>
-      </c>
-      <c r="L1" s="13" t="s">
-        <v>774</v>
       </c>
       <c r="M1" t="s">
         <v>727</v>
       </c>
       <c r="N1" s="13" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="O1" s="13" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="P1" s="13" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="Q1" s="13" t="s">
-        <v>770</v>
-      </c>
-    </row>
-    <row r="2" spans="1:17" ht="45" x14ac:dyDescent="0.25">
+        <v>769</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>28</v>
       </c>
       <c r="B2" t="s">
+        <v>761</v>
+      </c>
+      <c r="C2" t="s">
+        <v>763</v>
+      </c>
+      <c r="E2" s="12" t="s">
+        <v>777</v>
+      </c>
+      <c r="F2" t="s">
         <v>762</v>
-      </c>
-      <c r="C2" t="s">
-        <v>764</v>
-      </c>
-      <c r="E2" s="12" t="s">
-        <v>778</v>
-      </c>
-      <c r="F2" t="s">
-        <v>763</v>
       </c>
       <c r="G2">
         <v>7</v>
@@ -13585,36 +13645,36 @@
         <v>728</v>
       </c>
       <c r="L2" s="13" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="N2" s="13" t="s">
-        <v>791</v>
+        <v>790</v>
       </c>
       <c r="O2" s="13" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
       <c r="P2" s="13" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
       <c r="Q2" s="13" t="s">
-        <v>771</v>
-      </c>
-    </row>
-    <row r="3" spans="1:17" ht="45" x14ac:dyDescent="0.25">
+        <v>770</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>73</v>
       </c>
       <c r="B3" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
       <c r="C3" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="E3" s="12" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
       <c r="F3" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="G3">
         <v>18</v>
@@ -13629,33 +13689,33 @@
         <v>728</v>
       </c>
       <c r="L3" s="13" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="N3" s="13" t="s">
+        <v>767</v>
+      </c>
+      <c r="O3" s="13" t="s">
         <v>768</v>
       </c>
-      <c r="O3" s="13" t="s">
-        <v>769</v>
-      </c>
       <c r="P3" s="13" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
       <c r="Q3" s="13" t="s">
-        <v>771</v>
-      </c>
-    </row>
-    <row r="4" spans="1:17" ht="60" x14ac:dyDescent="0.25">
+        <v>770</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>150</v>
       </c>
       <c r="B4" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="E4" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
       <c r="F4" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="G4">
         <v>14</v>
@@ -13673,33 +13733,33 @@
         <v>424</v>
       </c>
       <c r="L4" s="13" t="s">
+        <v>782</v>
+      </c>
+      <c r="N4" s="13" t="s">
+        <v>767</v>
+      </c>
+      <c r="O4" s="13" t="s">
+        <v>781</v>
+      </c>
+      <c r="P4" s="13" t="s">
+        <v>780</v>
+      </c>
+      <c r="Q4" s="13" t="s">
         <v>783</v>
       </c>
-      <c r="N4" s="13" t="s">
-        <v>768</v>
-      </c>
-      <c r="O4" s="13" t="s">
-        <v>782</v>
-      </c>
-      <c r="P4" s="13" t="s">
-        <v>781</v>
-      </c>
-      <c r="Q4" s="13" t="s">
-        <v>784</v>
-      </c>
-    </row>
-    <row r="5" spans="1:17" ht="75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>206</v>
       </c>
       <c r="B5" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
       <c r="E5" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="F5" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="G5">
         <v>20</v>
@@ -13714,80 +13774,80 @@
         <v>8</v>
       </c>
       <c r="K5" s="13" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="L5" s="13" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="N5" s="13" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="O5" s="13" t="s">
+        <v>788</v>
+      </c>
+      <c r="P5" s="13" t="s">
         <v>789</v>
       </c>
-      <c r="P5" s="13" t="s">
-        <v>790</v>
-      </c>
       <c r="Q5" s="13" t="s">
-        <v>799</v>
-      </c>
-    </row>
-    <row r="6" spans="1:17" ht="60" x14ac:dyDescent="0.25">
+        <v>798</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>311</v>
       </c>
       <c r="B6" t="s">
+        <v>794</v>
+      </c>
+      <c r="C6" t="s">
         <v>795</v>
       </c>
-      <c r="C6" t="s">
-        <v>796</v>
-      </c>
       <c r="E6" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="F6" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
       <c r="G6">
         <v>12</v>
       </c>
       <c r="H6" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="I6">
         <v>6</v>
       </c>
       <c r="K6" s="13" t="s">
-        <v>910</v>
+        <v>909</v>
       </c>
       <c r="L6" s="13" t="s">
-        <v>823</v>
+        <v>822</v>
       </c>
       <c r="N6" s="13" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="O6" s="13" t="s">
+        <v>796</v>
+      </c>
+      <c r="P6" s="13" t="s">
         <v>797</v>
       </c>
-      <c r="P6" s="13" t="s">
-        <v>798</v>
-      </c>
       <c r="Q6" s="13" t="s">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="7" spans="1:17" ht="90" x14ac:dyDescent="0.25">
+        <v>799</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" ht="72" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>348</v>
       </c>
       <c r="B7" t="s">
+        <v>801</v>
+      </c>
+      <c r="E7" t="s">
         <v>802</v>
       </c>
-      <c r="E7" t="s">
-        <v>803</v>
-      </c>
       <c r="F7" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
       <c r="G7">
         <v>8</v>
@@ -13802,39 +13862,39 @@
         <v>4</v>
       </c>
       <c r="K7" s="13" t="s">
+        <v>806</v>
+      </c>
+      <c r="L7" s="13" t="s">
+        <v>805</v>
+      </c>
+      <c r="N7" s="13" t="s">
+        <v>767</v>
+      </c>
+      <c r="O7" s="13" t="s">
+        <v>803</v>
+      </c>
+      <c r="P7" s="13" t="s">
+        <v>804</v>
+      </c>
+      <c r="Q7" s="13" t="s">
         <v>807</v>
       </c>
-      <c r="L7" s="13" t="s">
-        <v>806</v>
-      </c>
-      <c r="N7" s="13" t="s">
-        <v>768</v>
-      </c>
-      <c r="O7" s="13" t="s">
-        <v>804</v>
-      </c>
-      <c r="P7" s="13" t="s">
-        <v>805</v>
-      </c>
-      <c r="Q7" s="13" t="s">
-        <v>808</v>
-      </c>
-    </row>
-    <row r="8" spans="1:17" ht="45" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:17" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>469</v>
       </c>
       <c r="B8" t="s">
+        <v>812</v>
+      </c>
+      <c r="C8" t="s">
         <v>813</v>
       </c>
-      <c r="C8" t="s">
-        <v>814</v>
-      </c>
       <c r="E8" t="s">
+        <v>809</v>
+      </c>
+      <c r="F8" t="s">
         <v>810</v>
-      </c>
-      <c r="F8" t="s">
-        <v>811</v>
       </c>
       <c r="G8">
         <v>30</v>
@@ -13852,33 +13912,33 @@
         <v>728</v>
       </c>
       <c r="L8" s="13" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
       <c r="N8" s="13" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="O8" s="13" t="s">
+        <v>814</v>
+      </c>
+      <c r="P8" s="13" t="s">
+        <v>811</v>
+      </c>
+      <c r="Q8" s="13" t="s">
         <v>815</v>
       </c>
-      <c r="P8" s="13" t="s">
-        <v>812</v>
-      </c>
-      <c r="Q8" s="13" t="s">
-        <v>816</v>
-      </c>
-    </row>
-    <row r="9" spans="1:17" ht="90" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:17" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>478</v>
       </c>
       <c r="B9" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
       <c r="E9" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="F9" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="G9">
         <v>41</v>
@@ -13893,33 +13953,33 @@
         <v>415</v>
       </c>
       <c r="L9" s="13" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
       <c r="N9" s="13" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="O9" s="13" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="P9" s="13" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
       <c r="Q9" s="13" t="s">
-        <v>821</v>
-      </c>
-    </row>
-    <row r="10" spans="1:17" ht="75" x14ac:dyDescent="0.25">
+        <v>820</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>483</v>
       </c>
       <c r="B10" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="E10" t="s">
-        <v>827</v>
+        <v>826</v>
       </c>
       <c r="F10" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
       <c r="G10">
         <v>143</v>
@@ -13931,30 +13991,30 @@
         <v>72</v>
       </c>
       <c r="K10" s="13" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="N10" s="13" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="O10" s="13" t="s">
+        <v>829</v>
+      </c>
+      <c r="P10" s="13" t="s">
         <v>830</v>
       </c>
-      <c r="P10" s="13" t="s">
-        <v>831</v>
-      </c>
-    </row>
-    <row r="11" spans="1:17" ht="60" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:17" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>529</v>
       </c>
       <c r="B11" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="E11" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
       <c r="F11" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="G11">
         <v>8</v>
@@ -13966,36 +14026,36 @@
         <v>2</v>
       </c>
       <c r="K11" s="13" t="s">
+        <v>836</v>
+      </c>
+      <c r="N11" s="13" t="s">
+        <v>767</v>
+      </c>
+      <c r="O11" s="13" t="s">
+        <v>834</v>
+      </c>
+      <c r="P11" s="13" t="s">
+        <v>833</v>
+      </c>
+      <c r="Q11" s="13" t="s">
         <v>837</v>
       </c>
-      <c r="N11" s="13" t="s">
-        <v>768</v>
-      </c>
-      <c r="O11" s="13" t="s">
-        <v>835</v>
-      </c>
-      <c r="P11" s="13" t="s">
-        <v>834</v>
-      </c>
-      <c r="Q11" s="13" t="s">
-        <v>838</v>
-      </c>
-    </row>
-    <row r="12" spans="1:17" ht="45" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:17" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>612</v>
       </c>
       <c r="B12" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="C12" t="s">
         <v>613</v>
       </c>
       <c r="E12" t="s">
+        <v>838</v>
+      </c>
+      <c r="F12" t="s">
         <v>839</v>
-      </c>
-      <c r="F12" t="s">
-        <v>840</v>
       </c>
       <c r="G12">
         <v>12</v>
@@ -14013,36 +14073,36 @@
         <v>424</v>
       </c>
       <c r="L12" s="13" t="s">
+        <v>842</v>
+      </c>
+      <c r="N12" s="13" t="s">
+        <v>767</v>
+      </c>
+      <c r="O12" s="13" t="s">
+        <v>841</v>
+      </c>
+      <c r="P12" s="13" t="s">
         <v>843</v>
       </c>
-      <c r="N12" s="13" t="s">
-        <v>768</v>
-      </c>
-      <c r="O12" s="13" t="s">
-        <v>842</v>
-      </c>
-      <c r="P12" s="13" t="s">
+      <c r="Q12" s="13" t="s">
         <v>844</v>
       </c>
-      <c r="Q12" s="13" t="s">
-        <v>845</v>
-      </c>
-    </row>
-    <row r="13" spans="1:17" ht="30" x14ac:dyDescent="0.25">
+    </row>
+    <row r="13" spans="1:17" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>617</v>
       </c>
       <c r="B13" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="C13" t="s">
         <v>618</v>
       </c>
       <c r="E13" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="F13" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
       <c r="G13">
         <v>24</v>
@@ -14057,36 +14117,36 @@
         <v>12</v>
       </c>
       <c r="K13" s="13" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="N13" s="13" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="O13" s="13" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="P13" s="13" t="s">
+        <v>852</v>
+      </c>
+      <c r="Q13" s="13" t="s">
         <v>853</v>
       </c>
-      <c r="Q13" s="13" t="s">
-        <v>854</v>
-      </c>
-    </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>621</v>
       </c>
       <c r="B14" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="C14" t="s">
         <v>622</v>
       </c>
       <c r="E14" s="12" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="F14" s="12" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="G14">
         <v>15</v>
@@ -14104,33 +14164,33 @@
         <v>424</v>
       </c>
       <c r="N14" s="13" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="O14" s="13" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="P14" s="13" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="Q14" s="13" t="s">
-        <v>855</v>
-      </c>
-    </row>
-    <row r="15" spans="1:17" ht="90" x14ac:dyDescent="0.25">
+        <v>854</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>625</v>
       </c>
       <c r="B15" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="C15" t="s">
         <v>626</v>
       </c>
       <c r="E15" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="F15" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
       <c r="G15">
         <v>6</v>
@@ -14145,33 +14205,33 @@
         <v>424</v>
       </c>
       <c r="M15" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="N15" s="13" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="O15" s="13" t="s">
+        <v>858</v>
+      </c>
+      <c r="P15" s="13" t="s">
         <v>859</v>
       </c>
-      <c r="P15" s="13" t="s">
+    </row>
+    <row r="16" spans="1:17" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
         <v>860</v>
       </c>
-    </row>
-    <row r="16" spans="1:17" ht="30" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+      <c r="B16" t="s">
+        <v>862</v>
+      </c>
+      <c r="C16" t="s">
+        <v>863</v>
+      </c>
+      <c r="E16" t="s">
+        <v>879</v>
+      </c>
+      <c r="F16" t="s">
         <v>861</v>
-      </c>
-      <c r="B16" t="s">
-        <v>863</v>
-      </c>
-      <c r="C16" t="s">
-        <v>864</v>
-      </c>
-      <c r="E16" t="s">
-        <v>880</v>
-      </c>
-      <c r="F16" t="s">
-        <v>862</v>
       </c>
       <c r="G16">
         <v>15</v>
@@ -14183,36 +14243,36 @@
         <v>3</v>
       </c>
       <c r="K16" s="13" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="L16" s="13" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
       <c r="M16" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
       <c r="N16" s="13" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="O16" s="13" t="s">
-        <v>877</v>
-      </c>
-    </row>
-    <row r="17" spans="1:17" ht="30" x14ac:dyDescent="0.25">
+        <v>876</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="B17" t="s">
+        <v>865</v>
+      </c>
+      <c r="C17" t="s">
         <v>866</v>
       </c>
-      <c r="C17" t="s">
-        <v>867</v>
-      </c>
       <c r="E17" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="F17" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
       <c r="G17">
         <v>48</v>
@@ -14227,36 +14287,36 @@
         <v>30</v>
       </c>
       <c r="K17" s="13" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="L17" s="13" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
       <c r="M17" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="N17" s="13" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="O17" s="13" t="s">
-        <v>842</v>
-      </c>
-    </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
+        <v>841</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
+        <v>868</v>
+      </c>
+      <c r="B18" t="s">
+        <v>870</v>
+      </c>
+      <c r="C18" t="s">
+        <v>871</v>
+      </c>
+      <c r="E18" t="s">
+        <v>872</v>
+      </c>
+      <c r="F18" s="12" t="s">
         <v>869</v>
-      </c>
-      <c r="B18" t="s">
-        <v>871</v>
-      </c>
-      <c r="C18" t="s">
-        <v>872</v>
-      </c>
-      <c r="E18" t="s">
-        <v>873</v>
-      </c>
-      <c r="F18" s="12" t="s">
-        <v>870</v>
       </c>
       <c r="G18">
         <v>8</v>
@@ -14274,30 +14334,30 @@
         <v>424</v>
       </c>
       <c r="M18" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="N18" s="13" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="O18" s="13" t="s">
-        <v>874</v>
-      </c>
-    </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
+        <v>873</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>629</v>
       </c>
       <c r="B19" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
       <c r="C19" t="s">
         <v>630</v>
       </c>
       <c r="E19" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
       <c r="F19" t="s">
-        <v>885</v>
+        <v>884</v>
       </c>
       <c r="G19">
         <v>9</v>
@@ -14315,33 +14375,33 @@
         <v>424</v>
       </c>
       <c r="N19" s="13" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="O19" s="13" t="s">
-        <v>886</v>
+        <v>885</v>
       </c>
       <c r="P19" s="13" t="s">
+        <v>887</v>
+      </c>
+      <c r="Q19" s="13" t="s">
         <v>888</v>
       </c>
-      <c r="Q19" s="13" t="s">
-        <v>889</v>
-      </c>
-    </row>
-    <row r="20" spans="1:17" ht="45" x14ac:dyDescent="0.25">
+    </row>
+    <row r="20" spans="1:17" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>633</v>
       </c>
       <c r="B20" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="C20" t="s">
         <v>634</v>
       </c>
       <c r="E20" t="s">
-        <v>894</v>
+        <v>893</v>
       </c>
       <c r="F20" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="G20">
         <v>8</v>
@@ -14353,36 +14413,36 @@
         <v>4</v>
       </c>
       <c r="K20" s="13" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
       <c r="L20" s="13" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
       <c r="N20" s="13" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="O20" s="13" t="s">
+        <v>890</v>
+      </c>
+      <c r="P20" s="13" t="s">
         <v>891</v>
       </c>
-      <c r="P20" s="13" t="s">
-        <v>892</v>
-      </c>
-    </row>
-    <row r="21" spans="1:17" ht="30" x14ac:dyDescent="0.25">
+    </row>
+    <row r="21" spans="1:17" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>637</v>
       </c>
       <c r="B21" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
       <c r="C21" t="s">
         <v>638</v>
       </c>
       <c r="E21" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
       <c r="F21" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
       <c r="G21">
         <v>166</v>
@@ -14400,30 +14460,30 @@
         <v>424</v>
       </c>
       <c r="N21" s="13" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="O21" s="13" t="s">
+        <v>898</v>
+      </c>
+      <c r="Q21" s="13" t="s">
         <v>899</v>
       </c>
-      <c r="Q21" s="13" t="s">
-        <v>900</v>
-      </c>
-    </row>
-    <row r="22" spans="1:17" ht="45" x14ac:dyDescent="0.25">
+    </row>
+    <row r="22" spans="1:17" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>708</v>
       </c>
       <c r="B22" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="C22" t="s">
         <v>709</v>
       </c>
       <c r="E22" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="F22" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="G22">
         <v>6</v>
@@ -14435,33 +14495,33 @@
         <v>4</v>
       </c>
       <c r="K22" s="13" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
       <c r="M22" t="s">
         <v>710</v>
       </c>
       <c r="N22" s="13" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="O22" s="13" t="s">
-        <v>903</v>
-      </c>
-    </row>
-    <row r="23" spans="1:17" ht="30" x14ac:dyDescent="0.25">
+        <v>902</v>
+      </c>
+    </row>
+    <row r="23" spans="1:17" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>713</v>
       </c>
       <c r="B23" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="C23" t="s">
         <v>714</v>
       </c>
       <c r="E23" t="s">
+        <v>905</v>
+      </c>
+      <c r="F23" t="s">
         <v>906</v>
-      </c>
-      <c r="F23" t="s">
-        <v>907</v>
       </c>
       <c r="G23">
         <v>36</v>
@@ -14476,189 +14536,360 @@
         <v>16</v>
       </c>
       <c r="K23" s="13" t="s">
-        <v>908</v>
+        <v>907</v>
       </c>
       <c r="M23" t="s">
         <v>715</v>
       </c>
       <c r="N23" s="13" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="O23" s="13" t="s">
-        <v>848</v>
-      </c>
-    </row>
-    <row r="24" spans="1:17" ht="30" x14ac:dyDescent="0.25">
+        <v>847</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17" ht="28.8" x14ac:dyDescent="0.3">
       <c r="D24" t="s">
         <v>641</v>
       </c>
-      <c r="F24" t="s">
+      <c r="E24" t="s">
+        <v>925</v>
+      </c>
+      <c r="F24" s="12" t="s">
         <v>734</v>
       </c>
       <c r="G24">
         <v>24</v>
       </c>
+      <c r="H24">
+        <v>15</v>
+      </c>
+      <c r="I24">
+        <v>9</v>
+      </c>
+      <c r="K24" s="13" t="s">
+        <v>913</v>
+      </c>
       <c r="L24" s="13" t="s">
-        <v>739</v>
+        <v>738</v>
+      </c>
+      <c r="N24" s="13" t="s">
+        <v>767</v>
+      </c>
+      <c r="O24" t="s">
+        <v>912</v>
       </c>
       <c r="P24" s="13" t="s">
-        <v>738</v>
-      </c>
-    </row>
-    <row r="25" spans="1:17" ht="45" x14ac:dyDescent="0.25">
+        <v>737</v>
+      </c>
+      <c r="Q24" s="13" t="s">
+        <v>926</v>
+      </c>
+    </row>
+    <row r="25" spans="1:17" ht="43.2" x14ac:dyDescent="0.3">
       <c r="D25" t="s">
         <v>645</v>
       </c>
-      <c r="F25" t="s">
+      <c r="E25" t="s">
+        <v>927</v>
+      </c>
+      <c r="F25" s="12" t="s">
         <v>735</v>
       </c>
       <c r="G25">
         <v>18</v>
       </c>
+      <c r="H25">
+        <v>6</v>
+      </c>
+      <c r="I25">
+        <v>3</v>
+      </c>
+      <c r="J25">
+        <v>9</v>
+      </c>
+      <c r="K25" s="13" t="s">
+        <v>928</v>
+      </c>
       <c r="L25" s="13" t="s">
-        <v>737</v>
+        <v>914</v>
+      </c>
+      <c r="N25" s="15" t="s">
+        <v>767</v>
+      </c>
+      <c r="O25" t="s">
+        <v>912</v>
       </c>
       <c r="P25" s="13" t="s">
         <v>736</v>
       </c>
     </row>
-    <row r="26" spans="1:17" ht="30" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:17" ht="100.8" x14ac:dyDescent="0.3">
       <c r="D26" t="s">
         <v>649</v>
       </c>
-      <c r="F26" t="s">
-        <v>740</v>
+      <c r="E26" t="s">
+        <v>929</v>
+      </c>
+      <c r="F26" s="12" t="s">
+        <v>739</v>
       </c>
       <c r="G26">
         <v>15</v>
       </c>
+      <c r="H26" t="s">
+        <v>931</v>
+      </c>
+      <c r="I26">
+        <v>9</v>
+      </c>
+      <c r="J26">
+        <v>6</v>
+      </c>
+      <c r="K26" s="13" t="s">
+        <v>930</v>
+      </c>
       <c r="L26" s="13" t="s">
-        <v>742</v>
+        <v>741</v>
+      </c>
+      <c r="N26" s="15" t="s">
+        <v>767</v>
+      </c>
+      <c r="O26" t="s">
+        <v>912</v>
       </c>
       <c r="P26" s="13" t="s">
-        <v>741</v>
-      </c>
-    </row>
-    <row r="27" spans="1:17" ht="75" x14ac:dyDescent="0.25">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="27" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
       <c r="D27" t="s">
         <v>653</v>
       </c>
+      <c r="E27" t="s">
+        <v>915</v>
+      </c>
       <c r="F27" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="G27">
         <v>24</v>
       </c>
+      <c r="H27">
+        <v>14</v>
+      </c>
+      <c r="I27">
+        <v>8</v>
+      </c>
+      <c r="K27" s="13" t="s">
+        <v>917</v>
+      </c>
       <c r="L27" s="13" t="s">
-        <v>745</v>
+        <v>744</v>
+      </c>
+      <c r="N27" s="15" t="s">
+        <v>767</v>
+      </c>
+      <c r="O27" t="s">
+        <v>916</v>
       </c>
       <c r="P27" s="13" t="s">
-        <v>744</v>
-      </c>
-    </row>
-    <row r="28" spans="1:17" ht="45" x14ac:dyDescent="0.25">
+        <v>743</v>
+      </c>
+    </row>
+    <row r="28" spans="1:17" ht="43.2" x14ac:dyDescent="0.3">
       <c r="D28" t="s">
         <v>657</v>
       </c>
+      <c r="E28" t="s">
+        <v>915</v>
+      </c>
       <c r="F28" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="G28">
         <v>27</v>
       </c>
+      <c r="H28">
+        <v>21</v>
+      </c>
+      <c r="I28">
+        <v>6</v>
+      </c>
+      <c r="K28" s="13" t="s">
+        <v>917</v>
+      </c>
       <c r="L28" s="13" t="s">
-        <v>748</v>
+        <v>747</v>
+      </c>
+      <c r="N28" s="15" t="s">
+        <v>767</v>
+      </c>
+      <c r="O28" t="s">
+        <v>916</v>
       </c>
       <c r="P28" s="13" t="s">
-        <v>747</v>
-      </c>
-    </row>
-    <row r="29" spans="1:17" ht="30" x14ac:dyDescent="0.25">
+        <v>746</v>
+      </c>
+    </row>
+    <row r="29" spans="1:17" ht="28.8" x14ac:dyDescent="0.3">
       <c r="D29" t="s">
         <v>661</v>
       </c>
+      <c r="E29" t="s">
+        <v>915</v>
+      </c>
       <c r="F29" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="G29">
         <v>24</v>
       </c>
+      <c r="H29" t="s">
+        <v>918</v>
+      </c>
       <c r="L29" s="13" t="s">
-        <v>745</v>
+        <v>744</v>
+      </c>
+      <c r="N29" s="15" t="s">
+        <v>767</v>
+      </c>
+      <c r="O29" t="s">
+        <v>916</v>
       </c>
       <c r="P29" s="13" t="s">
-        <v>750</v>
-      </c>
-    </row>
-    <row r="30" spans="1:17" ht="45" x14ac:dyDescent="0.25">
+        <v>749</v>
+      </c>
+    </row>
+    <row r="30" spans="1:17" ht="43.2" x14ac:dyDescent="0.3">
       <c r="D30" t="s">
         <v>665</v>
       </c>
+      <c r="E30" t="s">
+        <v>915</v>
+      </c>
       <c r="F30" s="12" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="G30">
         <v>9</v>
       </c>
+      <c r="H30">
+        <v>6</v>
+      </c>
+      <c r="I30">
+        <v>3</v>
+      </c>
       <c r="L30" s="13" t="s">
-        <v>745</v>
+        <v>744</v>
+      </c>
+      <c r="N30" s="15" t="s">
+        <v>767</v>
+      </c>
+      <c r="O30" t="s">
+        <v>916</v>
       </c>
       <c r="P30" s="13" t="s">
-        <v>752</v>
-      </c>
-    </row>
-    <row r="31" spans="1:17" x14ac:dyDescent="0.25">
+        <v>751</v>
+      </c>
+    </row>
+    <row r="31" spans="1:17" x14ac:dyDescent="0.3">
       <c r="D31" t="s">
         <v>669</v>
       </c>
+      <c r="E31" t="s">
+        <v>915</v>
+      </c>
       <c r="F31" t="s">
+        <v>752</v>
+      </c>
+      <c r="G31">
+        <v>9</v>
+      </c>
+      <c r="I31">
+        <v>3</v>
+      </c>
+      <c r="J31">
+        <v>6</v>
+      </c>
+      <c r="L31" s="13" t="s">
         <v>753</v>
       </c>
-      <c r="G31">
-        <v>18</v>
-      </c>
-      <c r="L31" s="13" t="s">
-        <v>754</v>
+      <c r="N31" s="15" t="s">
+        <v>767</v>
+      </c>
+      <c r="O31" s="13" t="s">
+        <v>916</v>
       </c>
       <c r="P31" s="14" t="s">
         <v>671</v>
       </c>
     </row>
-    <row r="32" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:17" x14ac:dyDescent="0.3">
       <c r="D32" t="s">
         <v>669</v>
       </c>
+      <c r="E32" t="s">
+        <v>915</v>
+      </c>
       <c r="F32" t="s">
+        <v>752</v>
+      </c>
+      <c r="G32">
+        <v>9</v>
+      </c>
+      <c r="I32">
+        <v>3</v>
+      </c>
+      <c r="J32">
+        <v>6</v>
+      </c>
+      <c r="L32" s="13" t="s">
         <v>753</v>
       </c>
-      <c r="G32">
-        <v>18</v>
-      </c>
-      <c r="L32" s="13" t="s">
-        <v>754</v>
+      <c r="N32" s="15" t="s">
+        <v>767</v>
+      </c>
+      <c r="O32" s="13" t="s">
+        <v>912</v>
       </c>
       <c r="P32" s="14" t="s">
         <v>673</v>
       </c>
     </row>
-    <row r="33" spans="4:16" ht="45" x14ac:dyDescent="0.25">
+    <row r="33" spans="4:16" ht="43.2" x14ac:dyDescent="0.3">
       <c r="D33" t="s">
         <v>675</v>
       </c>
+      <c r="E33" t="s">
+        <v>915</v>
+      </c>
       <c r="F33" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="G33">
         <v>21</v>
       </c>
+      <c r="H33">
+        <v>9</v>
+      </c>
+      <c r="I33">
+        <v>12</v>
+      </c>
       <c r="L33" s="13" t="s">
-        <v>748</v>
+        <v>747</v>
+      </c>
+      <c r="N33" s="15" t="s">
+        <v>767</v>
+      </c>
+      <c r="O33" s="13" t="s">
+        <v>916</v>
       </c>
       <c r="P33" s="13" t="s">
-        <v>747</v>
-      </c>
-    </row>
-    <row r="34" spans="4:16" x14ac:dyDescent="0.25">
+        <v>746</v>
+      </c>
+    </row>
+    <row r="34" spans="4:16" ht="57.6" x14ac:dyDescent="0.3">
       <c r="D34" t="s">
         <v>730</v>
       </c>
@@ -14668,14 +14899,29 @@
       <c r="G34">
         <v>27</v>
       </c>
+      <c r="H34">
+        <v>18</v>
+      </c>
+      <c r="I34">
+        <v>9</v>
+      </c>
+      <c r="K34" s="13" t="s">
+        <v>920</v>
+      </c>
       <c r="L34" s="13" t="s">
         <v>728</v>
       </c>
+      <c r="N34" s="15" t="s">
+        <v>767</v>
+      </c>
+      <c r="O34" s="13" t="s">
+        <v>919</v>
+      </c>
       <c r="P34" s="13" t="s">
         <v>731</v>
       </c>
     </row>
-    <row r="35" spans="4:16" x14ac:dyDescent="0.25">
+    <row r="35" spans="4:16" ht="57.6" x14ac:dyDescent="0.3">
       <c r="D35" t="s">
         <v>679</v>
       </c>
@@ -14685,105 +14931,183 @@
       <c r="G35">
         <v>36</v>
       </c>
+      <c r="H35">
+        <v>27</v>
+      </c>
+      <c r="I35">
+        <v>9</v>
+      </c>
+      <c r="K35" s="13" t="s">
+        <v>921</v>
+      </c>
       <c r="L35" s="13" t="s">
         <v>728</v>
       </c>
+      <c r="N35" s="15" t="s">
+        <v>767</v>
+      </c>
+      <c r="O35" s="13" t="s">
+        <v>916</v>
+      </c>
       <c r="P35" s="13" t="s">
         <v>729</v>
       </c>
     </row>
-    <row r="36" spans="4:16" x14ac:dyDescent="0.25">
+    <row r="36" spans="4:16" x14ac:dyDescent="0.3">
       <c r="D36" t="s">
         <v>683</v>
       </c>
       <c r="F36" t="s">
+        <v>755</v>
+      </c>
+      <c r="G36">
+        <v>6</v>
+      </c>
+      <c r="H36">
+        <v>3</v>
+      </c>
+      <c r="I36">
+        <v>3</v>
+      </c>
+      <c r="K36" s="13" t="s">
+        <v>728</v>
+      </c>
+      <c r="L36" s="13" t="s">
         <v>756</v>
       </c>
-      <c r="G36">
-        <v>12</v>
-      </c>
-      <c r="L36" s="13" t="s">
-        <v>757</v>
+      <c r="N36" s="15" t="s">
+        <v>767</v>
+      </c>
+      <c r="O36" t="s">
+        <v>923</v>
       </c>
       <c r="P36" s="13" t="s">
         <v>685</v>
       </c>
     </row>
-    <row r="37" spans="4:16" x14ac:dyDescent="0.25">
+    <row r="37" spans="4:16" x14ac:dyDescent="0.3">
       <c r="D37" t="s">
         <v>683</v>
       </c>
       <c r="F37" t="s">
+        <v>755</v>
+      </c>
+      <c r="G37">
+        <v>6</v>
+      </c>
+      <c r="H37">
+        <v>3</v>
+      </c>
+      <c r="I37">
+        <v>3</v>
+      </c>
+      <c r="K37" s="13" t="s">
+        <v>728</v>
+      </c>
+      <c r="L37" s="13" t="s">
         <v>756</v>
       </c>
-      <c r="G37">
-        <v>12</v>
-      </c>
-      <c r="L37" s="13" t="s">
-        <v>757</v>
+      <c r="N37" s="15" t="s">
+        <v>767</v>
+      </c>
+      <c r="O37" t="s">
+        <v>924</v>
       </c>
       <c r="P37" s="13" t="s">
         <v>687</v>
       </c>
     </row>
-    <row r="38" spans="4:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="38" spans="4:16" ht="28.8" x14ac:dyDescent="0.3">
       <c r="D38" t="s">
         <v>695</v>
       </c>
       <c r="F38" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="G38">
-        <v>8</v>
+        <v>4</v>
+      </c>
+      <c r="H38">
+        <v>4</v>
+      </c>
+      <c r="K38" s="13" t="s">
+        <v>922</v>
       </c>
       <c r="L38" s="13" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
       <c r="M38" t="s">
         <v>697</v>
       </c>
+      <c r="N38" s="15" t="s">
+        <v>767</v>
+      </c>
+      <c r="O38" s="13" t="s">
+        <v>916</v>
+      </c>
       <c r="P38" s="13" t="s">
-        <v>750</v>
-      </c>
-    </row>
-    <row r="39" spans="4:16" ht="30" x14ac:dyDescent="0.25">
+        <v>749</v>
+      </c>
+    </row>
+    <row r="39" spans="4:16" ht="28.8" x14ac:dyDescent="0.3">
       <c r="D39" t="s">
         <v>695</v>
       </c>
       <c r="F39" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="G39">
-        <v>8</v>
+        <v>4</v>
+      </c>
+      <c r="H39">
+        <v>4</v>
+      </c>
+      <c r="K39" s="13" t="s">
+        <v>922</v>
       </c>
       <c r="L39" s="13" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
       <c r="M39" t="s">
         <v>700</v>
       </c>
+      <c r="N39" s="15" t="s">
+        <v>767</v>
+      </c>
+      <c r="O39" s="13" t="s">
+        <v>916</v>
+      </c>
       <c r="P39" s="13" t="s">
-        <v>750</v>
-      </c>
-    </row>
-    <row r="40" spans="4:16" ht="30" x14ac:dyDescent="0.25">
+        <v>749</v>
+      </c>
+    </row>
+    <row r="40" spans="4:16" ht="28.8" x14ac:dyDescent="0.3">
       <c r="D40" t="s">
         <v>703</v>
       </c>
       <c r="F40" s="12" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="G40">
         <v>6</v>
       </c>
+      <c r="J40">
+        <v>6</v>
+      </c>
       <c r="L40" s="13" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="M40" t="s">
         <v>705</v>
       </c>
+      <c r="N40" s="15" t="s">
+        <v>767</v>
+      </c>
+      <c r="O40" s="13" t="s">
+        <v>916</v>
+      </c>
       <c r="P40" s="13" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
     </row>
   </sheetData>
@@ -14795,6 +15119,9 @@
     <hyperlink ref="F40" r:id="rId5" xr:uid="{3CE8ED52-391C-43D8-A8FA-F16C5BF55E1B}"/>
     <hyperlink ref="E3" r:id="rId6" xr:uid="{21C16D33-3989-405A-8D8C-EE7A7B101DC7}"/>
     <hyperlink ref="F30" r:id="rId7" xr:uid="{9DA84F45-BD83-4209-9C0F-6693193186A2}"/>
+    <hyperlink ref="F24" r:id="rId8" xr:uid="{60A42B3A-B33D-40F7-998C-BC0A6FDEEFEB}"/>
+    <hyperlink ref="F25" r:id="rId9" xr:uid="{B78CD678-227A-4045-BB40-438C2CB46B10}"/>
+    <hyperlink ref="F26" r:id="rId10" xr:uid="{61D7AE6D-7A01-4EA9-8013-8137F595E555}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>